<commit_message>
Fix swapped decode/prefill columns in 35B DLL comparison sheet
</commit_message>
<xml_diff>
--- a/data/snapdragon_llm_benchmarks_27B_35B.xlsx
+++ b/data/snapdragon_llm_benchmarks_27B_35B.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Andy\edgeAI_snapdragon\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Andy\Github\snapdragon-x2-elite-extreme-llm-benchmarks\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{64DA9C5D-AC19-4CE1-B784-F4EEAF66D46D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176265A2-AD4C-42E5-9D5E-8B7075E3CBF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QWEN_27B_Runs" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="QWEN_35B_Runs" sheetId="6" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -443,7 +442,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -513,20 +512,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1796,7 +1781,7 @@
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="33" t="s">
         <v>39</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -1837,7 +1822,7 @@
       <c r="O5" s="10"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="33" t="s">
         <v>39</v>
       </c>
       <c r="B6" s="6" t="s">
@@ -1878,7 +1863,7 @@
       <c r="O6" s="10"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="33" t="s">
         <v>39</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -1919,7 +1904,7 @@
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="33" t="s">
         <v>40</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -1960,7 +1945,7 @@
       <c r="O8" s="10"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A9" s="39" t="s">
+      <c r="A9" s="33" t="s">
         <v>40</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -2001,7 +1986,7 @@
       <c r="O9" s="10"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A10" s="39" t="s">
+      <c r="A10" s="33" t="s">
         <v>40</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -2042,7 +2027,7 @@
       <c r="O10" s="10"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="33" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -2083,7 +2068,7 @@
       <c r="O11" s="10"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="33" t="s">
         <v>41</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -2124,7 +2109,7 @@
       <c r="O12" s="10"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="33" t="s">
         <v>41</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -2165,7 +2150,7 @@
       <c r="O13" s="10"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A14" s="39" t="s">
+      <c r="A14" s="33" t="s">
         <v>42</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -2206,7 +2191,7 @@
       <c r="O14" s="10"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A15" s="39" t="s">
+      <c r="A15" s="33" t="s">
         <v>42</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -2247,7 +2232,7 @@
       <c r="O15" s="10"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A16" s="39" t="s">
+      <c r="A16" s="33" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="6" t="s">
@@ -2288,7 +2273,7 @@
       <c r="O16" s="10"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="33" t="s">
         <v>43</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -2329,7 +2314,7 @@
       <c r="O17" s="10"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A18" s="39" t="s">
+      <c r="A18" s="33" t="s">
         <v>43</v>
       </c>
       <c r="B18" s="6" t="s">
@@ -2370,7 +2355,7 @@
       <c r="O18" s="10"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A19" s="39" t="s">
+      <c r="A19" s="33" t="s">
         <v>43</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -2411,21 +2396,21 @@
       <c r="O19" s="10"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A20" s="33"/>
-      <c r="B20" s="34"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="34"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="35"/>
-      <c r="L20" s="34"/>
-      <c r="M20" s="36"/>
-      <c r="N20" s="37"/>
-      <c r="O20" s="38"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="23"/>
+      <c r="N20" s="24"/>
+      <c r="O20" s="25"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A21" s="20" t="s">
@@ -2447,7 +2432,7 @@
       <c r="O21" s="25"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A22" s="39" t="s">
+      <c r="A22" s="33" t="s">
         <v>44</v>
       </c>
       <c r="B22" s="32">
@@ -2488,7 +2473,7 @@
       <c r="O22" s="10"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A23" s="39" t="s">
+      <c r="A23" s="33" t="s">
         <v>44</v>
       </c>
       <c r="B23" s="32">
@@ -2529,7 +2514,7 @@
       <c r="O23" s="10"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A24" s="39" t="s">
+      <c r="A24" s="33" t="s">
         <v>44</v>
       </c>
       <c r="B24" s="32">
@@ -2570,7 +2555,7 @@
       <c r="O24" s="10"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A25" s="39" t="s">
+      <c r="A25" s="33" t="s">
         <v>45</v>
       </c>
       <c r="B25" s="32">
@@ -2611,7 +2596,7 @@
       <c r="O25" s="10"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A26" s="39" t="s">
+      <c r="A26" s="33" t="s">
         <v>45</v>
       </c>
       <c r="B26" s="32">
@@ -2652,7 +2637,7 @@
       <c r="O26" s="10"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A27" s="39" t="s">
+      <c r="A27" s="33" t="s">
         <v>45</v>
       </c>
       <c r="B27" s="32">
@@ -2693,7 +2678,7 @@
       <c r="O27" s="10"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A28" s="39" t="s">
+      <c r="A28" s="33" t="s">
         <v>46</v>
       </c>
       <c r="B28" s="32">
@@ -2734,7 +2719,7 @@
       <c r="O28" s="10"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A29" s="39" t="s">
+      <c r="A29" s="33" t="s">
         <v>46</v>
       </c>
       <c r="B29" s="32">
@@ -2775,7 +2760,7 @@
       <c r="O29" s="10"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A30" s="39" t="s">
+      <c r="A30" s="33" t="s">
         <v>46</v>
       </c>
       <c r="B30" s="32">
@@ -2816,7 +2801,7 @@
       <c r="O30" s="10"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A31" s="39" t="s">
+      <c r="A31" s="33" t="s">
         <v>47</v>
       </c>
       <c r="B31" s="32">
@@ -2857,7 +2842,7 @@
       <c r="O31" s="10"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="33" t="s">
         <v>47</v>
       </c>
       <c r="B32" s="32">
@@ -2898,7 +2883,7 @@
       <c r="O32" s="10"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A33" s="39" t="s">
+      <c r="A33" s="33" t="s">
         <v>47</v>
       </c>
       <c r="B33" s="32">
@@ -2939,7 +2924,7 @@
       <c r="O33" s="10"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A34" s="39" t="s">
+      <c r="A34" s="33" t="s">
         <v>48</v>
       </c>
       <c r="B34" s="32">
@@ -2980,7 +2965,7 @@
       <c r="O34" s="10"/>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A35" s="39" t="s">
+      <c r="A35" s="33" t="s">
         <v>48</v>
       </c>
       <c r="B35" s="32">
@@ -3021,7 +3006,7 @@
       <c r="O35" s="10"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A36" s="39" t="s">
+      <c r="A36" s="33" t="s">
         <v>48</v>
       </c>
       <c r="B36" s="32">
@@ -3079,7 +3064,7 @@
       <c r="O37" s="2"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A38" s="41" t="s">
+      <c r="A38" s="35" t="s">
         <v>51</v>
       </c>
       <c r="B38" s="2"/>
@@ -3098,7 +3083,7 @@
       <c r="O38" s="2"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A39" s="39" t="s">
+      <c r="A39" s="33" t="s">
         <v>49</v>
       </c>
       <c r="B39" s="6" t="s">
@@ -3131,7 +3116,7 @@
       <c r="K39" s="17">
         <v>0.91</v>
       </c>
-      <c r="L39" s="40" t="s">
+      <c r="L39" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M39" s="8"/>
@@ -3139,7 +3124,7 @@
       <c r="O39" s="10"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A40" s="39" t="s">
+      <c r="A40" s="33" t="s">
         <v>49</v>
       </c>
       <c r="B40" s="6" t="s">
@@ -3172,7 +3157,7 @@
       <c r="K40" s="17">
         <v>0.91</v>
       </c>
-      <c r="L40" s="40" t="s">
+      <c r="L40" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M40" s="8"/>
@@ -3180,7 +3165,7 @@
       <c r="O40" s="10"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A41" s="39" t="s">
+      <c r="A41" s="33" t="s">
         <v>49</v>
       </c>
       <c r="B41" s="6" t="s">
@@ -3213,7 +3198,7 @@
       <c r="K41" s="17">
         <v>0.91</v>
       </c>
-      <c r="L41" s="40" t="s">
+      <c r="L41" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M41" s="8"/>
@@ -3221,7 +3206,7 @@
       <c r="O41" s="10"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A42" s="39" t="s">
+      <c r="A42" s="33" t="s">
         <v>50</v>
       </c>
       <c r="B42" s="6" t="s">
@@ -3254,7 +3239,7 @@
       <c r="K42" s="17">
         <v>0.84</v>
       </c>
-      <c r="L42" s="40" t="s">
+      <c r="L42" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M42" s="8"/>
@@ -3262,7 +3247,7 @@
       <c r="O42" s="10"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A43" s="39" t="s">
+      <c r="A43" s="33" t="s">
         <v>50</v>
       </c>
       <c r="B43" s="6" t="s">
@@ -3295,7 +3280,7 @@
       <c r="K43" s="17">
         <v>0.84</v>
       </c>
-      <c r="L43" s="40" t="s">
+      <c r="L43" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M43" s="8"/>
@@ -3303,7 +3288,7 @@
       <c r="O43" s="10"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A44" s="39" t="s">
+      <c r="A44" s="33" t="s">
         <v>50</v>
       </c>
       <c r="B44" s="6" t="s">
@@ -3336,7 +3321,7 @@
       <c r="K44" s="17">
         <v>0.84</v>
       </c>
-      <c r="L44" s="40" t="s">
+      <c r="L44" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M44" s="8"/>
@@ -3344,7 +3329,7 @@
       <c r="O44" s="10"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A45" s="39" t="s">
+      <c r="A45" s="33" t="s">
         <v>52</v>
       </c>
       <c r="B45" s="6" t="s">
@@ -3377,7 +3362,7 @@
       <c r="K45" s="17">
         <v>0.79</v>
       </c>
-      <c r="L45" s="40" t="s">
+      <c r="L45" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M45" s="8"/>
@@ -3385,7 +3370,7 @@
       <c r="O45" s="10"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A46" s="39" t="s">
+      <c r="A46" s="33" t="s">
         <v>52</v>
       </c>
       <c r="B46" s="6" t="s">
@@ -3418,7 +3403,7 @@
       <c r="K46" s="17">
         <v>0.79</v>
       </c>
-      <c r="L46" s="40" t="s">
+      <c r="L46" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M46" s="8"/>
@@ -3426,7 +3411,7 @@
       <c r="O46" s="10"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A47" s="39" t="s">
+      <c r="A47" s="33" t="s">
         <v>52</v>
       </c>
       <c r="B47" s="6" t="s">
@@ -3459,7 +3444,7 @@
       <c r="K47" s="17">
         <v>0.79</v>
       </c>
-      <c r="L47" s="40" t="s">
+      <c r="L47" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M47" s="8"/>
@@ -3467,7 +3452,7 @@
       <c r="O47" s="10"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A48" s="39" t="s">
+      <c r="A48" s="33" t="s">
         <v>53</v>
       </c>
       <c r="B48" s="6" t="s">
@@ -3500,7 +3485,7 @@
       <c r="K48" s="17">
         <v>0.77</v>
       </c>
-      <c r="L48" s="40" t="s">
+      <c r="L48" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M48" s="8"/>
@@ -3508,7 +3493,7 @@
       <c r="O48" s="10"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A49" s="39" t="s">
+      <c r="A49" s="33" t="s">
         <v>53</v>
       </c>
       <c r="B49" s="6" t="s">
@@ -3541,7 +3526,7 @@
       <c r="K49" s="17">
         <v>0.77</v>
       </c>
-      <c r="L49" s="40" t="s">
+      <c r="L49" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M49" s="8"/>
@@ -3549,7 +3534,7 @@
       <c r="O49" s="10"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A50" s="39" t="s">
+      <c r="A50" s="33" t="s">
         <v>53</v>
       </c>
       <c r="B50" s="6" t="s">
@@ -3582,7 +3567,7 @@
       <c r="K50" s="17">
         <v>0.77</v>
       </c>
-      <c r="L50" s="40" t="s">
+      <c r="L50" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M50" s="8"/>
@@ -3590,7 +3575,7 @@
       <c r="O50" s="10"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A51" s="39" t="s">
+      <c r="A51" s="33" t="s">
         <v>54</v>
       </c>
       <c r="B51" s="6" t="s">
@@ -3623,7 +3608,7 @@
       <c r="K51" s="17">
         <v>0.69</v>
       </c>
-      <c r="L51" s="40" t="s">
+      <c r="L51" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M51" s="8"/>
@@ -3631,7 +3616,7 @@
       <c r="O51" s="10"/>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A52" s="39" t="s">
+      <c r="A52" s="33" t="s">
         <v>54</v>
       </c>
       <c r="B52" s="6" t="s">
@@ -3664,7 +3649,7 @@
       <c r="K52" s="17">
         <v>0.69</v>
       </c>
-      <c r="L52" s="40" t="s">
+      <c r="L52" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M52" s="8"/>
@@ -3672,7 +3657,7 @@
       <c r="O52" s="10"/>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A53" s="39" t="s">
+      <c r="A53" s="33" t="s">
         <v>54</v>
       </c>
       <c r="B53" s="6" t="s">
@@ -3705,7 +3690,7 @@
       <c r="K53" s="17">
         <v>0.69</v>
       </c>
-      <c r="L53" s="40" t="s">
+      <c r="L53" s="34" t="s">
         <v>25</v>
       </c>
       <c r="M53" s="8"/>
@@ -4423,10 +4408,10 @@
         <v>1</v>
       </c>
       <c r="I5" s="27">
+        <v>25.82</v>
+      </c>
+      <c r="J5" s="27">
         <v>412.75</v>
-      </c>
-      <c r="J5" s="27">
-        <v>25.82</v>
       </c>
       <c r="K5" s="28"/>
       <c r="L5" s="27" t="s">
@@ -4462,10 +4447,10 @@
         <v>3</v>
       </c>
       <c r="I6" s="27">
+        <v>28.04</v>
+      </c>
+      <c r="J6" s="27">
         <v>434.98</v>
-      </c>
-      <c r="J6" s="27">
-        <v>28.04</v>
       </c>
       <c r="K6" s="28"/>
       <c r="L6" s="27" t="s">
@@ -4501,10 +4486,10 @@
         <v>1</v>
       </c>
       <c r="I7" s="27">
+        <v>28.39</v>
+      </c>
+      <c r="J7" s="27">
         <v>463.09</v>
-      </c>
-      <c r="J7" s="27">
-        <v>28.39</v>
       </c>
       <c r="K7" s="28"/>
       <c r="L7" s="27" t="s">
@@ -4540,10 +4525,10 @@
         <v>3</v>
       </c>
       <c r="I8" s="27">
+        <v>28.48</v>
+      </c>
+      <c r="J8" s="27">
         <v>464.54</v>
-      </c>
-      <c r="J8" s="27">
-        <v>28.48</v>
       </c>
       <c r="K8" s="28"/>
       <c r="L8" s="27" t="s">

</xml_diff>